<commit_message>
Added Erstellt column, jira migrated to rest/api/3(from api/2)
</commit_message>
<xml_diff>
--- a/data/jira/OSIVnet Release Notes Template.xlsx
+++ b/data/jira/OSIVnet Release Notes Template.xlsx
@@ -11,7 +11,7 @@
     <sheet name="OSIVnet Release Notes" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'OSIVnet Release Notes'!$A$8:$F$8</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'OSIVnet Release Notes'!$A$8:$G$8</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t xml:space="preserve">Release</t>
   </si>
@@ -46,6 +46,9 @@
     <t xml:space="preserve">Komponente</t>
   </si>
   <si>
+    <t xml:space="preserve">Erstellt</t>
+  </si>
+  <si>
     <t xml:space="preserve">Geplant</t>
   </si>
   <si>
@@ -62,10 +65,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="@"/>
-    <numFmt numFmtId="166" formatCode="d/mm/yyyy"/>
+    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="166" formatCode="@"/>
+    <numFmt numFmtId="167" formatCode="d/mm/yyyy"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -163,12 +167,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="18">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -180,15 +188,19 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -198,6 +210,14 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -212,7 +232,11 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -256,9 +280,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>235080</xdr:colOff>
+      <xdr:colOff>233640</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>16200</xdr:rowOff>
+      <xdr:rowOff>14760</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -272,7 +296,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="3255120" cy="856800"/>
+          <a:ext cx="3253680" cy="855360"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -464,7 +488,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A2:F427"/>
+  <dimension ref="A2:G427"/>
   <sheetFormatPr defaultColWidth="11.43359375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.57"/>
@@ -472,1648 +496,1722 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="51.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="17.42"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="6" style="1" width="11.43"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="11.43"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="1" width="11.43"/>
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D2" s="2"/>
-      <c r="E2" s="3" t="s">
+      <c r="D2" s="3"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="G2" s="5" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F3" s="5" t="n">
+      <c r="F3" s="6"/>
+      <c r="G3" s="6" t="n">
         <v>45868</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="F8" s="8" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
+      <c r="G8" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="7"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="9"/>
-    </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="9"/>
-    </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7"/>
-      <c r="B11" s="7"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="9"/>
-    </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7"/>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="9"/>
-    </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7"/>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="9"/>
-    </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="9"/>
-    </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="s">
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="9"/>
-    </row>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7"/>
-      <c r="B16" s="7"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="9"/>
-    </row>
-    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7"/>
-      <c r="B17" s="7"/>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="9"/>
-    </row>
-    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7"/>
-      <c r="B18" s="7"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="9"/>
-    </row>
-    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7"/>
-      <c r="B19" s="7"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="9"/>
-    </row>
-    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7"/>
-      <c r="B20" s="7"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="9"/>
-    </row>
-    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7" t="s">
+      <c r="B9" s="9"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="12"/>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="9"/>
+      <c r="B10" s="9"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="12"/>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="9"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="12"/>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="9"/>
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="12"/>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="9"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="12"/>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="9"/>
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="13"/>
+      <c r="G14" s="12"/>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="B21" s="7"/>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="7"/>
-      <c r="F21" s="9"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="12"/>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="9"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="13"/>
+      <c r="G16" s="12"/>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="9"/>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="13"/>
+      <c r="G17" s="12"/>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="9"/>
+      <c r="B18" s="9"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="13"/>
+      <c r="G18" s="12"/>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="9"/>
+      <c r="B19" s="9"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="13"/>
+      <c r="G19" s="12"/>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="9"/>
+      <c r="B20" s="9"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="13"/>
+      <c r="G20" s="12"/>
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B21" s="9"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="13"/>
+      <c r="G21" s="12"/>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="7"/>
-      <c r="B22" s="7"/>
-      <c r="C22" s="7"/>
-      <c r="D22" s="7"/>
-      <c r="E22" s="7"/>
-      <c r="F22" s="9"/>
+      <c r="A22" s="9"/>
+      <c r="B22" s="9"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="13"/>
+      <c r="G22" s="12"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="10"/>
-      <c r="B23" s="10"/>
-      <c r="C23" s="10"/>
-      <c r="D23" s="10"/>
-      <c r="E23" s="10"/>
-      <c r="F23" s="11"/>
+      <c r="A23" s="14"/>
+      <c r="B23" s="14"/>
+      <c r="C23" s="14"/>
+      <c r="D23" s="14"/>
+      <c r="E23" s="14"/>
+      <c r="F23" s="15"/>
+      <c r="G23" s="16"/>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="10"/>
-      <c r="B24" s="10"/>
-      <c r="C24" s="10"/>
-      <c r="D24" s="10"/>
-      <c r="E24" s="10"/>
-      <c r="F24" s="11"/>
+      <c r="A24" s="14"/>
+      <c r="B24" s="14"/>
+      <c r="C24" s="14"/>
+      <c r="D24" s="14"/>
+      <c r="E24" s="14"/>
+      <c r="F24" s="15"/>
+      <c r="G24" s="16"/>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="10"/>
-      <c r="B25" s="10"/>
-      <c r="C25" s="10"/>
-      <c r="D25" s="10"/>
-      <c r="E25" s="10"/>
-      <c r="F25" s="11"/>
+      <c r="A25" s="14"/>
+      <c r="B25" s="14"/>
+      <c r="C25" s="14"/>
+      <c r="D25" s="14"/>
+      <c r="E25" s="14"/>
+      <c r="F25" s="15"/>
+      <c r="G25" s="16"/>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="10"/>
-      <c r="B26" s="10"/>
-      <c r="C26" s="10"/>
-      <c r="D26" s="10"/>
-      <c r="E26" s="10"/>
-      <c r="F26" s="11"/>
+      <c r="A26" s="14"/>
+      <c r="B26" s="14"/>
+      <c r="C26" s="14"/>
+      <c r="D26" s="14"/>
+      <c r="E26" s="14"/>
+      <c r="F26" s="15"/>
+      <c r="G26" s="16"/>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="10"/>
-      <c r="B27" s="10"/>
-      <c r="C27" s="10"/>
-      <c r="D27" s="10"/>
-      <c r="E27" s="10"/>
-      <c r="F27" s="11"/>
+      <c r="A27" s="14"/>
+      <c r="B27" s="14"/>
+      <c r="C27" s="14"/>
+      <c r="D27" s="14"/>
+      <c r="E27" s="14"/>
+      <c r="F27" s="15"/>
+      <c r="G27" s="16"/>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="10"/>
-      <c r="B28" s="10"/>
-      <c r="C28" s="10"/>
-      <c r="D28" s="10"/>
-      <c r="E28" s="10"/>
-      <c r="F28" s="11"/>
+      <c r="A28" s="14"/>
+      <c r="B28" s="14"/>
+      <c r="C28" s="14"/>
+      <c r="D28" s="14"/>
+      <c r="E28" s="14"/>
+      <c r="F28" s="15"/>
+      <c r="G28" s="16"/>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="10"/>
-      <c r="B29" s="10"/>
-      <c r="C29" s="10"/>
-      <c r="D29" s="10"/>
-      <c r="E29" s="10"/>
-      <c r="F29" s="11"/>
+      <c r="A29" s="14"/>
+      <c r="B29" s="14"/>
+      <c r="C29" s="14"/>
+      <c r="D29" s="14"/>
+      <c r="E29" s="14"/>
+      <c r="F29" s="15"/>
+      <c r="G29" s="16"/>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="10"/>
-      <c r="B30" s="10"/>
-      <c r="C30" s="10"/>
-      <c r="D30" s="10"/>
-      <c r="E30" s="10"/>
-      <c r="F30" s="11"/>
+      <c r="A30" s="14"/>
+      <c r="B30" s="14"/>
+      <c r="C30" s="14"/>
+      <c r="D30" s="14"/>
+      <c r="E30" s="14"/>
+      <c r="F30" s="15"/>
+      <c r="G30" s="16"/>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="10"/>
-      <c r="B31" s="10"/>
-      <c r="C31" s="10"/>
-      <c r="D31" s="10"/>
-      <c r="E31" s="10"/>
-      <c r="F31" s="11"/>
+      <c r="A31" s="14"/>
+      <c r="B31" s="14"/>
+      <c r="C31" s="14"/>
+      <c r="D31" s="14"/>
+      <c r="E31" s="14"/>
+      <c r="F31" s="15"/>
+      <c r="G31" s="16"/>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="10"/>
-      <c r="B32" s="10"/>
-      <c r="C32" s="10"/>
-      <c r="D32" s="10"/>
-      <c r="E32" s="10"/>
-      <c r="F32" s="11"/>
+      <c r="A32" s="14"/>
+      <c r="B32" s="14"/>
+      <c r="C32" s="14"/>
+      <c r="D32" s="14"/>
+      <c r="E32" s="14"/>
+      <c r="F32" s="15"/>
+      <c r="G32" s="16"/>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="10"/>
-      <c r="B33" s="10"/>
-      <c r="C33" s="10"/>
-      <c r="D33" s="10"/>
-      <c r="E33" s="10"/>
-      <c r="F33" s="11"/>
+      <c r="A33" s="14"/>
+      <c r="B33" s="14"/>
+      <c r="C33" s="14"/>
+      <c r="D33" s="14"/>
+      <c r="E33" s="14"/>
+      <c r="F33" s="15"/>
+      <c r="G33" s="16"/>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="10"/>
-      <c r="B34" s="10"/>
-      <c r="C34" s="10"/>
-      <c r="D34" s="10"/>
-      <c r="E34" s="10"/>
-      <c r="F34" s="11"/>
+      <c r="A34" s="14"/>
+      <c r="B34" s="14"/>
+      <c r="C34" s="14"/>
+      <c r="D34" s="14"/>
+      <c r="E34" s="14"/>
+      <c r="F34" s="15"/>
+      <c r="G34" s="16"/>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="10"/>
-      <c r="B35" s="10"/>
-      <c r="C35" s="10"/>
-      <c r="D35" s="10"/>
-      <c r="E35" s="10"/>
-      <c r="F35" s="11"/>
+      <c r="A35" s="14"/>
+      <c r="B35" s="14"/>
+      <c r="C35" s="14"/>
+      <c r="D35" s="14"/>
+      <c r="E35" s="14"/>
+      <c r="F35" s="15"/>
+      <c r="G35" s="16"/>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="10"/>
-      <c r="B36" s="10"/>
-      <c r="C36" s="10"/>
-      <c r="D36" s="10"/>
-      <c r="E36" s="10"/>
-      <c r="F36" s="11"/>
+      <c r="A36" s="14"/>
+      <c r="B36" s="14"/>
+      <c r="C36" s="14"/>
+      <c r="D36" s="14"/>
+      <c r="E36" s="14"/>
+      <c r="F36" s="15"/>
+      <c r="G36" s="16"/>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="10"/>
-      <c r="B37" s="10"/>
-      <c r="C37" s="10"/>
-      <c r="D37" s="10"/>
-      <c r="E37" s="10"/>
-      <c r="F37" s="11"/>
+      <c r="A37" s="14"/>
+      <c r="B37" s="14"/>
+      <c r="C37" s="14"/>
+      <c r="D37" s="14"/>
+      <c r="E37" s="14"/>
+      <c r="F37" s="15"/>
+      <c r="G37" s="16"/>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="10"/>
-      <c r="B38" s="10"/>
-      <c r="C38" s="10"/>
-      <c r="D38" s="10"/>
-      <c r="E38" s="10"/>
-      <c r="F38" s="11"/>
+      <c r="A38" s="14"/>
+      <c r="B38" s="14"/>
+      <c r="C38" s="14"/>
+      <c r="D38" s="14"/>
+      <c r="E38" s="14"/>
+      <c r="F38" s="15"/>
+      <c r="G38" s="16"/>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="10"/>
-      <c r="B39" s="10"/>
-      <c r="C39" s="10"/>
-      <c r="D39" s="10"/>
-      <c r="E39" s="10"/>
-      <c r="F39" s="11"/>
+      <c r="A39" s="14"/>
+      <c r="B39" s="14"/>
+      <c r="C39" s="14"/>
+      <c r="D39" s="14"/>
+      <c r="E39" s="14"/>
+      <c r="F39" s="15"/>
+      <c r="G39" s="16"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="10"/>
-      <c r="B40" s="10"/>
-      <c r="C40" s="10"/>
-      <c r="D40" s="10"/>
-      <c r="E40" s="10"/>
-      <c r="F40" s="11"/>
+      <c r="A40" s="14"/>
+      <c r="B40" s="14"/>
+      <c r="C40" s="14"/>
+      <c r="D40" s="14"/>
+      <c r="E40" s="14"/>
+      <c r="F40" s="15"/>
+      <c r="G40" s="16"/>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="10"/>
-      <c r="B41" s="10"/>
-      <c r="C41" s="10"/>
-      <c r="D41" s="10"/>
-      <c r="E41" s="10"/>
-      <c r="F41" s="11"/>
+      <c r="A41" s="14"/>
+      <c r="B41" s="14"/>
+      <c r="C41" s="14"/>
+      <c r="D41" s="14"/>
+      <c r="E41" s="14"/>
+      <c r="F41" s="15"/>
+      <c r="G41" s="16"/>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="10"/>
-      <c r="B42" s="10"/>
-      <c r="C42" s="10"/>
-      <c r="D42" s="10"/>
-      <c r="E42" s="10"/>
-      <c r="F42" s="11"/>
+      <c r="A42" s="14"/>
+      <c r="B42" s="14"/>
+      <c r="C42" s="14"/>
+      <c r="D42" s="14"/>
+      <c r="E42" s="14"/>
+      <c r="F42" s="15"/>
+      <c r="G42" s="16"/>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="10"/>
-      <c r="B43" s="10"/>
-      <c r="C43" s="10"/>
-      <c r="D43" s="10"/>
-      <c r="E43" s="10"/>
-      <c r="F43" s="11"/>
+      <c r="A43" s="14"/>
+      <c r="B43" s="14"/>
+      <c r="C43" s="14"/>
+      <c r="D43" s="14"/>
+      <c r="E43" s="14"/>
+      <c r="F43" s="15"/>
+      <c r="G43" s="16"/>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="10"/>
-      <c r="B44" s="10"/>
-      <c r="C44" s="10"/>
-      <c r="D44" s="10"/>
-      <c r="E44" s="10"/>
-      <c r="F44" s="11"/>
+      <c r="A44" s="14"/>
+      <c r="B44" s="14"/>
+      <c r="C44" s="14"/>
+      <c r="D44" s="14"/>
+      <c r="E44" s="14"/>
+      <c r="F44" s="15"/>
+      <c r="G44" s="16"/>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="10"/>
-      <c r="B45" s="10"/>
-      <c r="C45" s="10"/>
-      <c r="D45" s="10"/>
-      <c r="E45" s="10"/>
-      <c r="F45" s="11"/>
+      <c r="A45" s="14"/>
+      <c r="B45" s="14"/>
+      <c r="C45" s="14"/>
+      <c r="D45" s="14"/>
+      <c r="E45" s="14"/>
+      <c r="F45" s="15"/>
+      <c r="G45" s="16"/>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="10"/>
-      <c r="B46" s="10"/>
-      <c r="C46" s="10"/>
-      <c r="D46" s="10"/>
-      <c r="E46" s="10"/>
-      <c r="F46" s="11"/>
+      <c r="A46" s="14"/>
+      <c r="B46" s="14"/>
+      <c r="C46" s="14"/>
+      <c r="D46" s="14"/>
+      <c r="E46" s="14"/>
+      <c r="F46" s="15"/>
+      <c r="G46" s="16"/>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="10"/>
-      <c r="B47" s="10"/>
-      <c r="C47" s="10"/>
-      <c r="D47" s="10"/>
-      <c r="E47" s="10"/>
-      <c r="F47" s="11"/>
+      <c r="A47" s="14"/>
+      <c r="B47" s="14"/>
+      <c r="C47" s="14"/>
+      <c r="D47" s="14"/>
+      <c r="E47" s="14"/>
+      <c r="F47" s="15"/>
+      <c r="G47" s="16"/>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="10"/>
-      <c r="B48" s="10"/>
-      <c r="C48" s="10"/>
-      <c r="D48" s="10"/>
-      <c r="E48" s="10"/>
-      <c r="F48" s="11"/>
+      <c r="A48" s="14"/>
+      <c r="B48" s="14"/>
+      <c r="C48" s="14"/>
+      <c r="D48" s="14"/>
+      <c r="E48" s="14"/>
+      <c r="F48" s="15"/>
+      <c r="G48" s="16"/>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="10"/>
-      <c r="B49" s="10"/>
-      <c r="C49" s="10"/>
-      <c r="D49" s="10"/>
-      <c r="E49" s="10"/>
-      <c r="F49" s="11"/>
+      <c r="A49" s="14"/>
+      <c r="B49" s="14"/>
+      <c r="C49" s="14"/>
+      <c r="D49" s="14"/>
+      <c r="E49" s="14"/>
+      <c r="F49" s="15"/>
+      <c r="G49" s="16"/>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="10"/>
-      <c r="B50" s="10"/>
-      <c r="C50" s="10"/>
-      <c r="D50" s="10"/>
-      <c r="E50" s="10"/>
-      <c r="F50" s="11"/>
+      <c r="A50" s="14"/>
+      <c r="B50" s="14"/>
+      <c r="C50" s="14"/>
+      <c r="D50" s="14"/>
+      <c r="E50" s="14"/>
+      <c r="F50" s="15"/>
+      <c r="G50" s="16"/>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="10"/>
-      <c r="B51" s="10"/>
-      <c r="C51" s="10"/>
-      <c r="D51" s="10"/>
-      <c r="E51" s="10"/>
-      <c r="F51" s="11"/>
+      <c r="A51" s="14"/>
+      <c r="B51" s="14"/>
+      <c r="C51" s="14"/>
+      <c r="D51" s="14"/>
+      <c r="E51" s="14"/>
+      <c r="F51" s="15"/>
+      <c r="G51" s="16"/>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="10"/>
-      <c r="B52" s="10"/>
-      <c r="C52" s="10"/>
-      <c r="D52" s="10"/>
-      <c r="E52" s="10"/>
-      <c r="F52" s="11"/>
+      <c r="A52" s="14"/>
+      <c r="B52" s="14"/>
+      <c r="C52" s="14"/>
+      <c r="D52" s="14"/>
+      <c r="E52" s="14"/>
+      <c r="F52" s="15"/>
+      <c r="G52" s="16"/>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="10"/>
-      <c r="B53" s="10"/>
-      <c r="C53" s="10"/>
-      <c r="D53" s="10"/>
-      <c r="E53" s="10"/>
-      <c r="F53" s="11"/>
+      <c r="A53" s="14"/>
+      <c r="B53" s="14"/>
+      <c r="C53" s="14"/>
+      <c r="D53" s="14"/>
+      <c r="E53" s="14"/>
+      <c r="F53" s="15"/>
+      <c r="G53" s="16"/>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="10"/>
-      <c r="B54" s="10"/>
-      <c r="C54" s="10"/>
-      <c r="D54" s="10"/>
-      <c r="E54" s="10"/>
-      <c r="F54" s="11"/>
+      <c r="A54" s="14"/>
+      <c r="B54" s="14"/>
+      <c r="C54" s="14"/>
+      <c r="D54" s="14"/>
+      <c r="E54" s="14"/>
+      <c r="F54" s="15"/>
+      <c r="G54" s="16"/>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="10"/>
-      <c r="B55" s="10"/>
-      <c r="C55" s="10"/>
-      <c r="D55" s="10"/>
-      <c r="E55" s="10"/>
-      <c r="F55" s="11"/>
+      <c r="A55" s="14"/>
+      <c r="B55" s="14"/>
+      <c r="C55" s="14"/>
+      <c r="D55" s="14"/>
+      <c r="E55" s="14"/>
+      <c r="F55" s="15"/>
+      <c r="G55" s="16"/>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="10"/>
-      <c r="B56" s="10"/>
-      <c r="C56" s="10"/>
-      <c r="D56" s="10"/>
-      <c r="E56" s="10"/>
-      <c r="F56" s="11"/>
+      <c r="A56" s="14"/>
+      <c r="B56" s="14"/>
+      <c r="C56" s="14"/>
+      <c r="D56" s="14"/>
+      <c r="E56" s="14"/>
+      <c r="F56" s="15"/>
+      <c r="G56" s="16"/>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="10"/>
-      <c r="B57" s="10"/>
-      <c r="C57" s="10"/>
-      <c r="D57" s="10"/>
-      <c r="E57" s="10"/>
-      <c r="F57" s="11"/>
+      <c r="A57" s="14"/>
+      <c r="B57" s="14"/>
+      <c r="C57" s="14"/>
+      <c r="D57" s="14"/>
+      <c r="E57" s="14"/>
+      <c r="F57" s="15"/>
+      <c r="G57" s="16"/>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="10"/>
-      <c r="B58" s="10"/>
-      <c r="C58" s="10"/>
-      <c r="D58" s="10"/>
-      <c r="E58" s="10"/>
-      <c r="F58" s="11"/>
+      <c r="A58" s="14"/>
+      <c r="B58" s="14"/>
+      <c r="C58" s="14"/>
+      <c r="D58" s="14"/>
+      <c r="E58" s="14"/>
+      <c r="F58" s="15"/>
+      <c r="G58" s="16"/>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="10"/>
-      <c r="B59" s="10"/>
-      <c r="C59" s="10"/>
-      <c r="D59" s="10"/>
-      <c r="E59" s="10"/>
-      <c r="F59" s="11"/>
+      <c r="A59" s="14"/>
+      <c r="B59" s="14"/>
+      <c r="C59" s="14"/>
+      <c r="D59" s="14"/>
+      <c r="E59" s="14"/>
+      <c r="F59" s="15"/>
+      <c r="G59" s="16"/>
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="10"/>
-      <c r="B60" s="10"/>
-      <c r="C60" s="10"/>
-      <c r="D60" s="10"/>
-      <c r="E60" s="10"/>
-      <c r="F60" s="11"/>
+      <c r="A60" s="14"/>
+      <c r="B60" s="14"/>
+      <c r="C60" s="14"/>
+      <c r="D60" s="14"/>
+      <c r="E60" s="14"/>
+      <c r="F60" s="15"/>
+      <c r="G60" s="16"/>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="10"/>
-      <c r="B61" s="10"/>
-      <c r="C61" s="10"/>
-      <c r="D61" s="10"/>
-      <c r="E61" s="10"/>
-      <c r="F61" s="11"/>
+      <c r="A61" s="14"/>
+      <c r="B61" s="14"/>
+      <c r="C61" s="14"/>
+      <c r="D61" s="14"/>
+      <c r="E61" s="14"/>
+      <c r="F61" s="15"/>
+      <c r="G61" s="16"/>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="10"/>
-      <c r="B62" s="10"/>
-      <c r="C62" s="10"/>
-      <c r="D62" s="10"/>
-      <c r="E62" s="10"/>
-      <c r="F62" s="11"/>
+      <c r="A62" s="14"/>
+      <c r="B62" s="14"/>
+      <c r="C62" s="14"/>
+      <c r="D62" s="14"/>
+      <c r="E62" s="14"/>
+      <c r="F62" s="15"/>
+      <c r="G62" s="16"/>
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="10"/>
-      <c r="B63" s="10"/>
-      <c r="C63" s="10"/>
-      <c r="D63" s="10"/>
-      <c r="E63" s="10"/>
-      <c r="F63" s="11"/>
+      <c r="A63" s="14"/>
+      <c r="B63" s="14"/>
+      <c r="C63" s="14"/>
+      <c r="D63" s="14"/>
+      <c r="E63" s="14"/>
+      <c r="F63" s="15"/>
+      <c r="G63" s="16"/>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="10"/>
-      <c r="B64" s="10"/>
-      <c r="C64" s="10"/>
-      <c r="D64" s="10"/>
-      <c r="E64" s="10"/>
-      <c r="F64" s="11"/>
+      <c r="A64" s="14"/>
+      <c r="B64" s="14"/>
+      <c r="C64" s="14"/>
+      <c r="D64" s="14"/>
+      <c r="E64" s="14"/>
+      <c r="F64" s="15"/>
+      <c r="G64" s="16"/>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="10"/>
-      <c r="B65" s="10"/>
-      <c r="C65" s="10"/>
-      <c r="D65" s="10"/>
-      <c r="E65" s="10"/>
-      <c r="F65" s="11"/>
+      <c r="A65" s="14"/>
+      <c r="B65" s="14"/>
+      <c r="C65" s="14"/>
+      <c r="D65" s="14"/>
+      <c r="E65" s="14"/>
+      <c r="F65" s="15"/>
+      <c r="G65" s="16"/>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="10"/>
-      <c r="B66" s="10"/>
-      <c r="C66" s="10"/>
-      <c r="D66" s="10"/>
-      <c r="E66" s="10"/>
-      <c r="F66" s="11"/>
+      <c r="A66" s="14"/>
+      <c r="B66" s="14"/>
+      <c r="C66" s="14"/>
+      <c r="D66" s="14"/>
+      <c r="E66" s="14"/>
+      <c r="F66" s="15"/>
+      <c r="G66" s="16"/>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="10"/>
-      <c r="B67" s="10"/>
-      <c r="C67" s="10"/>
-      <c r="D67" s="10"/>
-      <c r="E67" s="10"/>
-      <c r="F67" s="11"/>
+      <c r="A67" s="14"/>
+      <c r="B67" s="14"/>
+      <c r="C67" s="14"/>
+      <c r="D67" s="14"/>
+      <c r="E67" s="14"/>
+      <c r="F67" s="15"/>
+      <c r="G67" s="16"/>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="10"/>
-      <c r="B68" s="10"/>
-      <c r="C68" s="10"/>
-      <c r="D68" s="10"/>
-      <c r="E68" s="10"/>
-      <c r="F68" s="11"/>
+      <c r="A68" s="14"/>
+      <c r="B68" s="14"/>
+      <c r="C68" s="14"/>
+      <c r="D68" s="14"/>
+      <c r="E68" s="14"/>
+      <c r="F68" s="15"/>
+      <c r="G68" s="16"/>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="10"/>
-      <c r="B69" s="10"/>
-      <c r="C69" s="10"/>
-      <c r="D69" s="10"/>
-      <c r="E69" s="10"/>
-      <c r="F69" s="11"/>
+      <c r="A69" s="14"/>
+      <c r="B69" s="14"/>
+      <c r="C69" s="14"/>
+      <c r="D69" s="14"/>
+      <c r="E69" s="14"/>
+      <c r="F69" s="15"/>
+      <c r="G69" s="16"/>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="10"/>
-      <c r="B70" s="10"/>
-      <c r="C70" s="10"/>
-      <c r="D70" s="10"/>
-      <c r="E70" s="10"/>
-      <c r="F70" s="11"/>
+      <c r="A70" s="14"/>
+      <c r="B70" s="14"/>
+      <c r="C70" s="14"/>
+      <c r="D70" s="14"/>
+      <c r="E70" s="14"/>
+      <c r="F70" s="15"/>
+      <c r="G70" s="16"/>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="10"/>
-      <c r="B71" s="10"/>
-      <c r="C71" s="10"/>
-      <c r="D71" s="10"/>
-      <c r="E71" s="10"/>
-      <c r="F71" s="11"/>
+      <c r="A71" s="14"/>
+      <c r="B71" s="14"/>
+      <c r="C71" s="14"/>
+      <c r="D71" s="14"/>
+      <c r="E71" s="14"/>
+      <c r="F71" s="15"/>
+      <c r="G71" s="16"/>
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="10"/>
-      <c r="B72" s="10"/>
-      <c r="C72" s="10"/>
-      <c r="D72" s="10"/>
-      <c r="E72" s="10"/>
-      <c r="F72" s="11"/>
+      <c r="A72" s="14"/>
+      <c r="B72" s="14"/>
+      <c r="C72" s="14"/>
+      <c r="D72" s="14"/>
+      <c r="E72" s="14"/>
+      <c r="F72" s="15"/>
+      <c r="G72" s="16"/>
     </row>
     <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="10"/>
-      <c r="B73" s="10"/>
-      <c r="C73" s="10"/>
-      <c r="D73" s="10"/>
-      <c r="E73" s="10"/>
-      <c r="F73" s="11"/>
+      <c r="A73" s="14"/>
+      <c r="B73" s="14"/>
+      <c r="C73" s="14"/>
+      <c r="D73" s="14"/>
+      <c r="E73" s="14"/>
+      <c r="F73" s="15"/>
+      <c r="G73" s="16"/>
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="10"/>
-      <c r="B74" s="10"/>
-      <c r="C74" s="10"/>
-      <c r="D74" s="10"/>
-      <c r="E74" s="10"/>
-      <c r="F74" s="11"/>
+      <c r="A74" s="14"/>
+      <c r="B74" s="14"/>
+      <c r="C74" s="14"/>
+      <c r="D74" s="14"/>
+      <c r="E74" s="14"/>
+      <c r="F74" s="15"/>
+      <c r="G74" s="16"/>
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="10"/>
-      <c r="B75" s="10"/>
-      <c r="C75" s="10"/>
-      <c r="D75" s="10"/>
-      <c r="E75" s="10"/>
-      <c r="F75" s="11"/>
+      <c r="A75" s="14"/>
+      <c r="B75" s="14"/>
+      <c r="C75" s="14"/>
+      <c r="D75" s="14"/>
+      <c r="E75" s="14"/>
+      <c r="F75" s="15"/>
+      <c r="G75" s="16"/>
     </row>
     <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="10"/>
-      <c r="B76" s="10"/>
-      <c r="C76" s="10"/>
-      <c r="D76" s="10"/>
-      <c r="E76" s="10"/>
-      <c r="F76" s="11"/>
+      <c r="A76" s="14"/>
+      <c r="B76" s="14"/>
+      <c r="C76" s="14"/>
+      <c r="D76" s="14"/>
+      <c r="E76" s="14"/>
+      <c r="F76" s="15"/>
+      <c r="G76" s="16"/>
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F77" s="12"/>
+      <c r="G77" s="17"/>
     </row>
     <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F78" s="12"/>
+      <c r="G78" s="17"/>
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F79" s="12"/>
+      <c r="G79" s="17"/>
     </row>
     <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F80" s="12"/>
+      <c r="G80" s="17"/>
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F81" s="12"/>
+      <c r="G81" s="17"/>
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F82" s="12"/>
+      <c r="G82" s="17"/>
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F83" s="12"/>
+      <c r="G83" s="17"/>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F84" s="12"/>
+      <c r="G84" s="17"/>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F85" s="12"/>
+      <c r="G85" s="17"/>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F86" s="12"/>
+      <c r="G86" s="17"/>
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F87" s="12"/>
+      <c r="G87" s="17"/>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F88" s="12"/>
+      <c r="G88" s="17"/>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F89" s="12"/>
+      <c r="G89" s="17"/>
     </row>
     <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F90" s="12"/>
+      <c r="G90" s="17"/>
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F91" s="12"/>
+      <c r="G91" s="17"/>
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F92" s="12"/>
+      <c r="G92" s="17"/>
     </row>
     <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F93" s="12"/>
+      <c r="G93" s="17"/>
     </row>
     <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F94" s="12"/>
+      <c r="G94" s="17"/>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F95" s="12"/>
+      <c r="G95" s="17"/>
     </row>
     <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F96" s="12"/>
+      <c r="G96" s="17"/>
     </row>
     <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F97" s="12"/>
+      <c r="G97" s="17"/>
     </row>
     <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F98" s="12"/>
+      <c r="G98" s="17"/>
     </row>
     <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F99" s="12"/>
+      <c r="G99" s="17"/>
     </row>
     <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F100" s="12"/>
+      <c r="G100" s="17"/>
     </row>
     <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F101" s="12"/>
+      <c r="G101" s="17"/>
     </row>
     <row r="102" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F102" s="12"/>
+      <c r="G102" s="17"/>
     </row>
     <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F103" s="12"/>
+      <c r="G103" s="17"/>
     </row>
     <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F104" s="12"/>
+      <c r="G104" s="17"/>
     </row>
     <row r="105" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F105" s="12"/>
+      <c r="G105" s="17"/>
     </row>
     <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F106" s="12"/>
+      <c r="G106" s="17"/>
     </row>
     <row r="107" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F107" s="12"/>
+      <c r="G107" s="17"/>
     </row>
     <row r="108" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F108" s="12"/>
+      <c r="G108" s="17"/>
     </row>
     <row r="109" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F109" s="12"/>
+      <c r="G109" s="17"/>
     </row>
     <row r="110" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F110" s="12"/>
+      <c r="G110" s="17"/>
     </row>
     <row r="111" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F111" s="12"/>
+      <c r="G111" s="17"/>
     </row>
     <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F112" s="12"/>
+      <c r="G112" s="17"/>
     </row>
     <row r="113" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F113" s="12"/>
+      <c r="G113" s="17"/>
     </row>
     <row r="114" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F114" s="12"/>
+      <c r="G114" s="17"/>
     </row>
     <row r="115" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F115" s="12"/>
+      <c r="G115" s="17"/>
     </row>
     <row r="116" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F116" s="12"/>
+      <c r="G116" s="17"/>
     </row>
     <row r="117" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F117" s="12"/>
+      <c r="G117" s="17"/>
     </row>
     <row r="118" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F118" s="12"/>
+      <c r="G118" s="17"/>
     </row>
     <row r="119" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F119" s="12"/>
+      <c r="G119" s="17"/>
     </row>
     <row r="120" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F120" s="12"/>
+      <c r="G120" s="17"/>
     </row>
     <row r="121" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F121" s="12"/>
+      <c r="G121" s="17"/>
     </row>
     <row r="122" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F122" s="12"/>
+      <c r="G122" s="17"/>
     </row>
     <row r="123" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F123" s="12"/>
+      <c r="G123" s="17"/>
     </row>
     <row r="124" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F124" s="12"/>
+      <c r="G124" s="17"/>
     </row>
     <row r="125" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F125" s="12"/>
+      <c r="G125" s="17"/>
     </row>
     <row r="126" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F126" s="12"/>
+      <c r="G126" s="17"/>
     </row>
     <row r="127" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F127" s="12"/>
+      <c r="G127" s="17"/>
     </row>
     <row r="128" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F128" s="12"/>
+      <c r="G128" s="17"/>
     </row>
     <row r="129" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F129" s="12"/>
+      <c r="G129" s="17"/>
     </row>
     <row r="130" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F130" s="12"/>
+      <c r="G130" s="17"/>
     </row>
     <row r="131" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F131" s="12"/>
+      <c r="G131" s="17"/>
     </row>
     <row r="132" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F132" s="12"/>
+      <c r="G132" s="17"/>
     </row>
     <row r="133" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F133" s="12"/>
+      <c r="G133" s="17"/>
     </row>
     <row r="134" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F134" s="12"/>
+      <c r="G134" s="17"/>
     </row>
     <row r="135" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F135" s="12"/>
+      <c r="G135" s="17"/>
     </row>
     <row r="136" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F136" s="12"/>
+      <c r="G136" s="17"/>
     </row>
     <row r="137" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F137" s="12"/>
+      <c r="G137" s="17"/>
     </row>
     <row r="138" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F138" s="12"/>
+      <c r="G138" s="17"/>
     </row>
     <row r="139" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F139" s="12"/>
+      <c r="G139" s="17"/>
     </row>
     <row r="140" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F140" s="12"/>
+      <c r="G140" s="17"/>
     </row>
     <row r="141" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F141" s="12"/>
+      <c r="G141" s="17"/>
     </row>
     <row r="142" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F142" s="12"/>
+      <c r="G142" s="17"/>
     </row>
     <row r="143" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F143" s="12"/>
+      <c r="G143" s="17"/>
     </row>
     <row r="144" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F144" s="12"/>
+      <c r="G144" s="17"/>
     </row>
     <row r="145" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F145" s="12"/>
+      <c r="G145" s="17"/>
     </row>
     <row r="146" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F146" s="12"/>
+      <c r="G146" s="17"/>
     </row>
     <row r="147" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F147" s="12"/>
+      <c r="G147" s="17"/>
     </row>
     <row r="148" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F148" s="12"/>
+      <c r="G148" s="17"/>
     </row>
     <row r="149" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F149" s="12"/>
+      <c r="G149" s="17"/>
     </row>
     <row r="150" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F150" s="12"/>
+      <c r="G150" s="17"/>
     </row>
     <row r="151" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F151" s="12"/>
+      <c r="G151" s="17"/>
     </row>
     <row r="152" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F152" s="12"/>
+      <c r="G152" s="17"/>
     </row>
     <row r="153" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F153" s="12"/>
+      <c r="G153" s="17"/>
     </row>
     <row r="154" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F154" s="12"/>
+      <c r="G154" s="17"/>
     </row>
     <row r="155" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F155" s="12"/>
+      <c r="G155" s="17"/>
     </row>
     <row r="156" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F156" s="12"/>
+      <c r="G156" s="17"/>
     </row>
     <row r="157" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F157" s="12"/>
+      <c r="G157" s="17"/>
     </row>
     <row r="158" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F158" s="12"/>
+      <c r="G158" s="17"/>
     </row>
     <row r="159" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F159" s="12"/>
+      <c r="G159" s="17"/>
     </row>
     <row r="160" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F160" s="12"/>
+      <c r="G160" s="17"/>
     </row>
     <row r="161" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F161" s="12"/>
+      <c r="G161" s="17"/>
     </row>
     <row r="162" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F162" s="12"/>
+      <c r="G162" s="17"/>
     </row>
     <row r="163" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F163" s="12"/>
+      <c r="G163" s="17"/>
     </row>
     <row r="164" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F164" s="12"/>
+      <c r="G164" s="17"/>
     </row>
     <row r="165" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F165" s="12"/>
+      <c r="G165" s="17"/>
     </row>
     <row r="166" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F166" s="12"/>
+      <c r="G166" s="17"/>
     </row>
     <row r="167" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F167" s="12"/>
+      <c r="G167" s="17"/>
     </row>
     <row r="168" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F168" s="12"/>
+      <c r="G168" s="17"/>
     </row>
     <row r="169" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F169" s="12"/>
+      <c r="G169" s="17"/>
     </row>
     <row r="170" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F170" s="12"/>
+      <c r="G170" s="17"/>
     </row>
     <row r="171" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F171" s="12"/>
+      <c r="G171" s="17"/>
     </row>
     <row r="172" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F172" s="12"/>
+      <c r="G172" s="17"/>
     </row>
     <row r="173" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F173" s="12"/>
+      <c r="G173" s="17"/>
     </row>
     <row r="174" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F174" s="12"/>
+      <c r="G174" s="17"/>
     </row>
     <row r="175" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F175" s="12"/>
+      <c r="G175" s="17"/>
     </row>
     <row r="176" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F176" s="12"/>
+      <c r="G176" s="17"/>
     </row>
     <row r="177" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F177" s="12"/>
+      <c r="G177" s="17"/>
     </row>
     <row r="178" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F178" s="12"/>
+      <c r="G178" s="17"/>
     </row>
     <row r="179" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F179" s="12"/>
+      <c r="G179" s="17"/>
     </row>
     <row r="180" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F180" s="12"/>
+      <c r="G180" s="17"/>
     </row>
     <row r="181" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F181" s="12"/>
+      <c r="G181" s="17"/>
     </row>
     <row r="182" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F182" s="12"/>
+      <c r="G182" s="17"/>
     </row>
     <row r="183" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F183" s="12"/>
+      <c r="G183" s="17"/>
     </row>
     <row r="184" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F184" s="12"/>
+      <c r="G184" s="17"/>
     </row>
     <row r="185" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F185" s="12"/>
+      <c r="G185" s="17"/>
     </row>
     <row r="186" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F186" s="12"/>
+      <c r="G186" s="17"/>
     </row>
     <row r="187" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F187" s="12"/>
+      <c r="G187" s="17"/>
     </row>
     <row r="188" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F188" s="12"/>
+      <c r="G188" s="17"/>
     </row>
     <row r="189" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F189" s="12"/>
+      <c r="G189" s="17"/>
     </row>
     <row r="190" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F190" s="12"/>
+      <c r="G190" s="17"/>
     </row>
     <row r="191" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F191" s="12"/>
+      <c r="G191" s="17"/>
     </row>
     <row r="192" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F192" s="12"/>
+      <c r="G192" s="17"/>
     </row>
     <row r="193" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F193" s="12"/>
+      <c r="G193" s="17"/>
     </row>
     <row r="194" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F194" s="12"/>
+      <c r="G194" s="17"/>
     </row>
     <row r="195" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F195" s="12"/>
+      <c r="G195" s="17"/>
     </row>
     <row r="196" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F196" s="12"/>
+      <c r="G196" s="17"/>
     </row>
     <row r="197" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F197" s="12"/>
+      <c r="G197" s="17"/>
     </row>
     <row r="198" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F198" s="12"/>
+      <c r="G198" s="17"/>
     </row>
     <row r="199" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F199" s="12"/>
+      <c r="G199" s="17"/>
     </row>
     <row r="200" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F200" s="12"/>
+      <c r="G200" s="17"/>
     </row>
     <row r="201" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F201" s="12"/>
+      <c r="G201" s="17"/>
     </row>
     <row r="202" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F202" s="12"/>
+      <c r="G202" s="17"/>
     </row>
     <row r="203" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F203" s="12"/>
+      <c r="G203" s="17"/>
     </row>
     <row r="204" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F204" s="12"/>
+      <c r="G204" s="17"/>
     </row>
     <row r="205" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F205" s="12"/>
+      <c r="G205" s="17"/>
     </row>
     <row r="206" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F206" s="12"/>
+      <c r="G206" s="17"/>
     </row>
     <row r="207" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F207" s="12"/>
+      <c r="G207" s="17"/>
     </row>
     <row r="208" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F208" s="12"/>
+      <c r="G208" s="17"/>
     </row>
     <row r="209" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F209" s="12"/>
+      <c r="G209" s="17"/>
     </row>
     <row r="210" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F210" s="12"/>
+      <c r="G210" s="17"/>
     </row>
     <row r="211" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F211" s="12"/>
+      <c r="G211" s="17"/>
     </row>
     <row r="212" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F212" s="12"/>
+      <c r="G212" s="17"/>
     </row>
     <row r="213" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F213" s="12"/>
+      <c r="G213" s="17"/>
     </row>
     <row r="214" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F214" s="12"/>
+      <c r="G214" s="17"/>
     </row>
     <row r="215" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F215" s="12"/>
+      <c r="G215" s="17"/>
     </row>
     <row r="216" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F216" s="12"/>
+      <c r="G216" s="17"/>
     </row>
     <row r="217" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F217" s="12"/>
+      <c r="G217" s="17"/>
     </row>
     <row r="218" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F218" s="12"/>
+      <c r="G218" s="17"/>
     </row>
     <row r="219" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F219" s="12"/>
+      <c r="G219" s="17"/>
     </row>
     <row r="220" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F220" s="12"/>
+      <c r="G220" s="17"/>
     </row>
     <row r="221" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F221" s="12"/>
+      <c r="G221" s="17"/>
     </row>
     <row r="222" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F222" s="12"/>
+      <c r="G222" s="17"/>
     </row>
     <row r="223" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F223" s="12"/>
+      <c r="G223" s="17"/>
     </row>
     <row r="224" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F224" s="12"/>
+      <c r="G224" s="17"/>
     </row>
     <row r="225" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F225" s="12"/>
+      <c r="G225" s="17"/>
     </row>
     <row r="226" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F226" s="12"/>
+      <c r="G226" s="17"/>
     </row>
     <row r="227" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F227" s="12"/>
+      <c r="G227" s="17"/>
     </row>
     <row r="228" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F228" s="12"/>
+      <c r="G228" s="17"/>
     </row>
     <row r="229" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F229" s="12"/>
+      <c r="G229" s="17"/>
     </row>
     <row r="230" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F230" s="12"/>
+      <c r="G230" s="17"/>
     </row>
     <row r="231" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F231" s="12"/>
+      <c r="G231" s="17"/>
     </row>
     <row r="232" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F232" s="12"/>
+      <c r="G232" s="17"/>
     </row>
     <row r="233" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F233" s="12"/>
+      <c r="G233" s="17"/>
     </row>
     <row r="234" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F234" s="12"/>
+      <c r="G234" s="17"/>
     </row>
     <row r="235" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F235" s="12"/>
+      <c r="G235" s="17"/>
     </row>
     <row r="236" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F236" s="12"/>
+      <c r="G236" s="17"/>
     </row>
     <row r="237" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F237" s="12"/>
+      <c r="G237" s="17"/>
     </row>
     <row r="238" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F238" s="12"/>
+      <c r="G238" s="17"/>
     </row>
     <row r="239" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F239" s="12"/>
+      <c r="G239" s="17"/>
     </row>
     <row r="240" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F240" s="12"/>
+      <c r="G240" s="17"/>
     </row>
     <row r="241" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F241" s="12"/>
+      <c r="G241" s="17"/>
     </row>
     <row r="242" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F242" s="12"/>
+      <c r="G242" s="17"/>
     </row>
     <row r="243" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F243" s="12"/>
+      <c r="G243" s="17"/>
     </row>
     <row r="244" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F244" s="12"/>
+      <c r="G244" s="17"/>
     </row>
     <row r="245" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F245" s="12"/>
+      <c r="G245" s="17"/>
     </row>
     <row r="246" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F246" s="12"/>
+      <c r="G246" s="17"/>
     </row>
     <row r="247" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F247" s="12"/>
+      <c r="G247" s="17"/>
     </row>
     <row r="248" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F248" s="12"/>
+      <c r="G248" s="17"/>
     </row>
     <row r="249" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F249" s="12"/>
+      <c r="G249" s="17"/>
     </row>
     <row r="250" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F250" s="12"/>
+      <c r="G250" s="17"/>
     </row>
     <row r="251" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F251" s="12"/>
+      <c r="G251" s="17"/>
     </row>
     <row r="252" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F252" s="12"/>
+      <c r="G252" s="17"/>
     </row>
     <row r="253" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F253" s="12"/>
+      <c r="G253" s="17"/>
     </row>
     <row r="254" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F254" s="12"/>
+      <c r="G254" s="17"/>
     </row>
     <row r="255" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F255" s="12"/>
+      <c r="G255" s="17"/>
     </row>
     <row r="256" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F256" s="12"/>
+      <c r="G256" s="17"/>
     </row>
     <row r="257" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F257" s="12"/>
+      <c r="G257" s="17"/>
     </row>
     <row r="258" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F258" s="12"/>
+      <c r="G258" s="17"/>
     </row>
     <row r="259" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F259" s="12"/>
+      <c r="G259" s="17"/>
     </row>
     <row r="260" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F260" s="12"/>
+      <c r="G260" s="17"/>
     </row>
     <row r="261" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F261" s="12"/>
+      <c r="G261" s="17"/>
     </row>
     <row r="262" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F262" s="12"/>
+      <c r="G262" s="17"/>
     </row>
     <row r="263" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F263" s="12"/>
+      <c r="G263" s="17"/>
     </row>
     <row r="264" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F264" s="12"/>
+      <c r="G264" s="17"/>
     </row>
     <row r="265" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F265" s="12"/>
+      <c r="G265" s="17"/>
     </row>
     <row r="266" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F266" s="12"/>
+      <c r="G266" s="17"/>
     </row>
     <row r="267" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F267" s="12"/>
+      <c r="G267" s="17"/>
     </row>
     <row r="268" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F268" s="12"/>
+      <c r="G268" s="17"/>
     </row>
     <row r="269" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F269" s="12"/>
+      <c r="G269" s="17"/>
     </row>
     <row r="270" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F270" s="12"/>
+      <c r="G270" s="17"/>
     </row>
     <row r="271" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F271" s="12"/>
+      <c r="G271" s="17"/>
     </row>
     <row r="272" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F272" s="12"/>
+      <c r="G272" s="17"/>
     </row>
     <row r="273" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F273" s="12"/>
+      <c r="G273" s="17"/>
     </row>
     <row r="274" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F274" s="12"/>
+      <c r="G274" s="17"/>
     </row>
     <row r="275" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F275" s="12"/>
+      <c r="G275" s="17"/>
     </row>
     <row r="276" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F276" s="12"/>
+      <c r="G276" s="17"/>
     </row>
     <row r="277" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F277" s="12"/>
+      <c r="G277" s="17"/>
     </row>
     <row r="278" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F278" s="12"/>
+      <c r="G278" s="17"/>
     </row>
     <row r="279" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F279" s="12"/>
+      <c r="G279" s="17"/>
     </row>
     <row r="280" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F280" s="12"/>
+      <c r="G280" s="17"/>
     </row>
     <row r="281" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F281" s="12"/>
+      <c r="G281" s="17"/>
     </row>
     <row r="282" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F282" s="12"/>
+      <c r="G282" s="17"/>
     </row>
     <row r="283" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F283" s="12"/>
+      <c r="G283" s="17"/>
     </row>
     <row r="284" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F284" s="12"/>
+      <c r="G284" s="17"/>
     </row>
     <row r="285" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F285" s="12"/>
+      <c r="G285" s="17"/>
     </row>
     <row r="286" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F286" s="12"/>
+      <c r="G286" s="17"/>
     </row>
     <row r="287" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F287" s="12"/>
+      <c r="G287" s="17"/>
     </row>
     <row r="288" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F288" s="12"/>
+      <c r="G288" s="17"/>
     </row>
     <row r="289" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F289" s="12"/>
+      <c r="G289" s="17"/>
     </row>
     <row r="290" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F290" s="12"/>
+      <c r="G290" s="17"/>
     </row>
     <row r="291" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F291" s="12"/>
+      <c r="G291" s="17"/>
     </row>
     <row r="292" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F292" s="12"/>
+      <c r="G292" s="17"/>
     </row>
     <row r="293" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F293" s="12"/>
+      <c r="G293" s="17"/>
     </row>
     <row r="294" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F294" s="12"/>
+      <c r="G294" s="17"/>
     </row>
     <row r="295" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F295" s="12"/>
+      <c r="G295" s="17"/>
     </row>
     <row r="296" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F296" s="12"/>
+      <c r="G296" s="17"/>
     </row>
     <row r="297" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F297" s="12"/>
+      <c r="G297" s="17"/>
     </row>
     <row r="298" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F298" s="12"/>
+      <c r="G298" s="17"/>
     </row>
     <row r="299" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F299" s="12"/>
+      <c r="G299" s="17"/>
     </row>
     <row r="300" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F300" s="12"/>
+      <c r="G300" s="17"/>
     </row>
     <row r="301" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F301" s="12"/>
+      <c r="G301" s="17"/>
     </row>
     <row r="302" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F302" s="12"/>
+      <c r="G302" s="17"/>
     </row>
     <row r="303" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F303" s="12"/>
+      <c r="G303" s="17"/>
     </row>
     <row r="304" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F304" s="12"/>
+      <c r="G304" s="17"/>
     </row>
     <row r="305" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F305" s="12"/>
+      <c r="G305" s="17"/>
     </row>
     <row r="306" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F306" s="12"/>
+      <c r="G306" s="17"/>
     </row>
     <row r="307" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F307" s="12"/>
+      <c r="G307" s="17"/>
     </row>
     <row r="308" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F308" s="12"/>
+      <c r="G308" s="17"/>
     </row>
     <row r="309" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F309" s="12"/>
+      <c r="G309" s="17"/>
     </row>
     <row r="310" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F310" s="12"/>
+      <c r="G310" s="17"/>
     </row>
     <row r="311" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F311" s="12"/>
+      <c r="G311" s="17"/>
     </row>
     <row r="312" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F312" s="12"/>
+      <c r="G312" s="17"/>
     </row>
     <row r="313" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F313" s="12"/>
+      <c r="G313" s="17"/>
     </row>
     <row r="314" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F314" s="12"/>
+      <c r="G314" s="17"/>
     </row>
     <row r="315" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F315" s="12"/>
+      <c r="G315" s="17"/>
     </row>
     <row r="316" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F316" s="12"/>
+      <c r="G316" s="17"/>
     </row>
     <row r="317" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F317" s="12"/>
+      <c r="G317" s="17"/>
     </row>
     <row r="318" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F318" s="12"/>
+      <c r="G318" s="17"/>
     </row>
     <row r="319" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F319" s="12"/>
+      <c r="G319" s="17"/>
     </row>
     <row r="320" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F320" s="12"/>
+      <c r="G320" s="17"/>
     </row>
     <row r="321" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F321" s="12"/>
+      <c r="G321" s="17"/>
     </row>
     <row r="322" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F322" s="12"/>
+      <c r="G322" s="17"/>
     </row>
     <row r="323" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F323" s="12"/>
+      <c r="G323" s="17"/>
     </row>
     <row r="324" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F324" s="12"/>
+      <c r="G324" s="17"/>
     </row>
     <row r="325" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F325" s="12"/>
+      <c r="G325" s="17"/>
     </row>
     <row r="326" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F326" s="12"/>
+      <c r="G326" s="17"/>
     </row>
     <row r="327" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F327" s="12"/>
+      <c r="G327" s="17"/>
     </row>
     <row r="328" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F328" s="12"/>
+      <c r="G328" s="17"/>
     </row>
     <row r="329" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F329" s="12"/>
+      <c r="G329" s="17"/>
     </row>
     <row r="330" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F330" s="12"/>
+      <c r="G330" s="17"/>
     </row>
     <row r="331" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F331" s="12"/>
+      <c r="G331" s="17"/>
     </row>
     <row r="332" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F332" s="12"/>
+      <c r="G332" s="17"/>
     </row>
     <row r="333" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F333" s="12"/>
+      <c r="G333" s="17"/>
     </row>
     <row r="334" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F334" s="12"/>
+      <c r="G334" s="17"/>
     </row>
     <row r="335" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F335" s="12"/>
+      <c r="G335" s="17"/>
     </row>
     <row r="336" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F336" s="12"/>
+      <c r="G336" s="17"/>
     </row>
     <row r="337" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F337" s="12"/>
+      <c r="G337" s="17"/>
     </row>
     <row r="338" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F338" s="12"/>
+      <c r="G338" s="17"/>
     </row>
     <row r="339" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F339" s="12"/>
+      <c r="G339" s="17"/>
     </row>
     <row r="340" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F340" s="12"/>
+      <c r="G340" s="17"/>
     </row>
     <row r="341" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F341" s="12"/>
+      <c r="G341" s="17"/>
     </row>
     <row r="342" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F342" s="12"/>
+      <c r="G342" s="17"/>
     </row>
     <row r="343" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F343" s="12"/>
+      <c r="G343" s="17"/>
     </row>
     <row r="344" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F344" s="12"/>
+      <c r="G344" s="17"/>
     </row>
     <row r="345" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F345" s="12"/>
+      <c r="G345" s="17"/>
     </row>
     <row r="346" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F346" s="12"/>
+      <c r="G346" s="17"/>
     </row>
     <row r="347" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F347" s="12"/>
+      <c r="G347" s="17"/>
     </row>
     <row r="348" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F348" s="12"/>
+      <c r="G348" s="17"/>
     </row>
     <row r="349" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F349" s="12"/>
+      <c r="G349" s="17"/>
     </row>
     <row r="350" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F350" s="12"/>
+      <c r="G350" s="17"/>
     </row>
     <row r="351" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F351" s="12"/>
+      <c r="G351" s="17"/>
     </row>
     <row r="352" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F352" s="12"/>
+      <c r="G352" s="17"/>
     </row>
     <row r="353" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F353" s="12"/>
+      <c r="G353" s="17"/>
     </row>
     <row r="354" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F354" s="12"/>
+      <c r="G354" s="17"/>
     </row>
     <row r="355" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F355" s="12"/>
+      <c r="G355" s="17"/>
     </row>
     <row r="356" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F356" s="12"/>
+      <c r="G356" s="17"/>
     </row>
     <row r="357" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F357" s="12"/>
+      <c r="G357" s="17"/>
     </row>
     <row r="358" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F358" s="12"/>
+      <c r="G358" s="17"/>
     </row>
     <row r="359" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F359" s="12"/>
+      <c r="G359" s="17"/>
     </row>
     <row r="360" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F360" s="12"/>
+      <c r="G360" s="17"/>
     </row>
     <row r="361" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F361" s="12"/>
+      <c r="G361" s="17"/>
     </row>
     <row r="362" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F362" s="12"/>
+      <c r="G362" s="17"/>
     </row>
     <row r="363" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F363" s="12"/>
+      <c r="G363" s="17"/>
     </row>
     <row r="364" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F364" s="12"/>
+      <c r="G364" s="17"/>
     </row>
     <row r="365" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F365" s="12"/>
+      <c r="G365" s="17"/>
     </row>
     <row r="366" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F366" s="12"/>
+      <c r="G366" s="17"/>
     </row>
     <row r="367" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F367" s="12"/>
+      <c r="G367" s="17"/>
     </row>
     <row r="368" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F368" s="12"/>
+      <c r="G368" s="17"/>
     </row>
     <row r="369" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F369" s="12"/>
+      <c r="G369" s="17"/>
     </row>
     <row r="370" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F370" s="12"/>
+      <c r="G370" s="17"/>
     </row>
     <row r="371" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F371" s="12"/>
+      <c r="G371" s="17"/>
     </row>
     <row r="372" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F372" s="12"/>
+      <c r="G372" s="17"/>
     </row>
     <row r="373" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F373" s="12"/>
+      <c r="G373" s="17"/>
     </row>
     <row r="374" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F374" s="12"/>
+      <c r="G374" s="17"/>
     </row>
     <row r="375" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F375" s="12"/>
+      <c r="G375" s="17"/>
     </row>
     <row r="376" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F376" s="12"/>
+      <c r="G376" s="17"/>
     </row>
     <row r="377" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F377" s="12"/>
+      <c r="G377" s="17"/>
     </row>
     <row r="378" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F378" s="12"/>
+      <c r="G378" s="17"/>
     </row>
     <row r="379" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F379" s="12"/>
+      <c r="G379" s="17"/>
     </row>
     <row r="380" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F380" s="12"/>
+      <c r="G380" s="17"/>
     </row>
     <row r="381" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F381" s="12"/>
+      <c r="G381" s="17"/>
     </row>
     <row r="382" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F382" s="12"/>
+      <c r="G382" s="17"/>
     </row>
     <row r="383" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F383" s="12"/>
+      <c r="G383" s="17"/>
     </row>
     <row r="384" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F384" s="12"/>
+      <c r="G384" s="17"/>
     </row>
     <row r="385" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F385" s="12"/>
+      <c r="G385" s="17"/>
     </row>
     <row r="386" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F386" s="12"/>
+      <c r="G386" s="17"/>
     </row>
     <row r="387" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F387" s="12"/>
+      <c r="G387" s="17"/>
     </row>
     <row r="388" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F388" s="12"/>
+      <c r="G388" s="17"/>
     </row>
     <row r="389" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F389" s="12"/>
+      <c r="G389" s="17"/>
     </row>
     <row r="390" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F390" s="12"/>
+      <c r="G390" s="17"/>
     </row>
     <row r="391" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F391" s="12"/>
+      <c r="G391" s="17"/>
     </row>
     <row r="392" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F392" s="12"/>
+      <c r="G392" s="17"/>
     </row>
     <row r="393" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F393" s="12"/>
+      <c r="G393" s="17"/>
     </row>
     <row r="394" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F394" s="12"/>
+      <c r="G394" s="17"/>
     </row>
     <row r="395" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F395" s="12"/>
+      <c r="G395" s="17"/>
     </row>
     <row r="396" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F396" s="12"/>
+      <c r="G396" s="17"/>
     </row>
     <row r="397" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F397" s="12"/>
+      <c r="G397" s="17"/>
     </row>
     <row r="398" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F398" s="12"/>
+      <c r="G398" s="17"/>
     </row>
     <row r="399" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F399" s="12"/>
+      <c r="G399" s="17"/>
     </row>
     <row r="400" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F400" s="12"/>
+      <c r="G400" s="17"/>
     </row>
     <row r="401" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F401" s="12"/>
+      <c r="G401" s="17"/>
     </row>
     <row r="402" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F402" s="12"/>
+      <c r="G402" s="17"/>
     </row>
     <row r="403" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F403" s="12"/>
+      <c r="G403" s="17"/>
     </row>
     <row r="404" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F404" s="12"/>
+      <c r="G404" s="17"/>
     </row>
     <row r="405" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F405" s="12"/>
+      <c r="G405" s="17"/>
     </row>
     <row r="406" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F406" s="12"/>
+      <c r="G406" s="17"/>
     </row>
     <row r="407" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F407" s="12"/>
+      <c r="G407" s="17"/>
     </row>
     <row r="408" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F408" s="12"/>
+      <c r="G408" s="17"/>
     </row>
     <row r="409" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F409" s="12"/>
+      <c r="G409" s="17"/>
     </row>
     <row r="410" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F410" s="12"/>
+      <c r="G410" s="17"/>
     </row>
     <row r="411" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F411" s="12"/>
+      <c r="G411" s="17"/>
     </row>
     <row r="412" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F412" s="12"/>
+      <c r="G412" s="17"/>
     </row>
     <row r="413" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F413" s="12"/>
+      <c r="G413" s="17"/>
     </row>
     <row r="414" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F414" s="12"/>
+      <c r="G414" s="17"/>
     </row>
     <row r="415" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F415" s="12"/>
+      <c r="G415" s="17"/>
     </row>
     <row r="416" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F416" s="12"/>
+      <c r="G416" s="17"/>
     </row>
     <row r="417" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F417" s="12"/>
+      <c r="G417" s="17"/>
     </row>
     <row r="418" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F418" s="12"/>
+      <c r="G418" s="17"/>
     </row>
     <row r="419" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F419" s="12"/>
+      <c r="G419" s="17"/>
     </row>
     <row r="420" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F420" s="12"/>
+      <c r="G420" s="17"/>
     </row>
     <row r="421" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F421" s="12"/>
+      <c r="G421" s="17"/>
     </row>
     <row r="422" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F422" s="12"/>
+      <c r="G422" s="17"/>
     </row>
     <row r="423" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F423" s="12"/>
+      <c r="G423" s="17"/>
     </row>
     <row r="424" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F424" s="12"/>
+      <c r="G424" s="17"/>
     </row>
     <row r="425" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F425" s="12"/>
+      <c r="G425" s="17"/>
     </row>
     <row r="426" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F426" s="12"/>
+      <c r="G426" s="17"/>
     </row>
     <row r="427" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F427" s="12"/>
+      <c r="G427" s="17"/>
     </row>
   </sheetData>
-  <autoFilter ref="A8:F8"/>
+  <autoFilter ref="A8:G8"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.39375" right="0.39375" top="0.39375" bottom="0.39375" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>